<commit_message>
vault backup: 2024-03-12 12:15:55
</commit_message>
<xml_diff>
--- a/public/assets/excel_router_solution.xlsx
+++ b/public/assets/excel_router_solution.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marcc\git\informatikgarten.ch\public\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63F6059B-5C28-4A34-A909-D724F5B28683}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{119D18B8-AA1F-4464-BA40-4B39E3A68C67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="14220" activeTab="2" xr2:uid="{8B4C5CB2-983E-4FDC-89E4-8A1111F2665D}"/>
+    <workbookView minimized="1" xWindow="930" yWindow="2110" windowWidth="14180" windowHeight="11600" activeTab="1" xr2:uid="{8B4C5CB2-983E-4FDC-89E4-8A1111F2665D}"/>
   </bookViews>
   <sheets>
     <sheet name="Einstieg" sheetId="1" r:id="rId1"/>
@@ -1643,13 +1643,13 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>530413</xdr:colOff>
+      <xdr:colOff>530415</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>173868</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>698510</xdr:colOff>
+      <xdr:colOff>610578</xdr:colOff>
       <xdr:row>30</xdr:row>
       <xdr:rowOff>75595</xdr:rowOff>
     </xdr:to>
@@ -1666,10 +1666,10 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="5754044" y="362856"/>
-          <a:ext cx="2443514" cy="5465537"/>
+          <a:off x="5761838" y="364368"/>
+          <a:ext cx="2371048" cy="5509265"/>
           <a:chOff x="5754044" y="362856"/>
-          <a:chExt cx="2443514" cy="5397501"/>
+          <a:chExt cx="2482335" cy="5397501"/>
         </a:xfrm>
       </xdr:grpSpPr>
       <xdr:sp macro="" textlink="">
@@ -1685,8 +1685,8 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
-            <a:off x="5835952" y="362856"/>
-            <a:ext cx="2281128" cy="5397501"/>
+            <a:off x="5835951" y="362856"/>
+            <a:ext cx="2400428" cy="5397501"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -3614,10 +3614,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
@@ -5425,7 +5421,7 @@
         <v>255</v>
       </c>
       <c r="U10" s="11" t="str">
-        <f>DEC2BIN(T10,8)</f>
+        <f t="shared" ref="U10:U18" si="1">DEC2BIN(T10,8)</f>
         <v>11111111</v>
       </c>
       <c r="V10" s="11"/>
@@ -5492,7 +5488,7 @@
         <v>254</v>
       </c>
       <c r="U11" s="11" t="str">
-        <f>DEC2BIN(T11,8)</f>
+        <f t="shared" si="1"/>
         <v>11111110</v>
       </c>
       <c r="V11" s="11"/>
@@ -5520,7 +5516,7 @@
         <v>252</v>
       </c>
       <c r="U12" s="11" t="str">
-        <f>DEC2BIN(T12,8)</f>
+        <f t="shared" si="1"/>
         <v>11111100</v>
       </c>
       <c r="V12" s="11"/>
@@ -5549,7 +5545,7 @@
         <v>248</v>
       </c>
       <c r="U13" s="11" t="str">
-        <f>DEC2BIN(T13,8)</f>
+        <f t="shared" si="1"/>
         <v>11111000</v>
       </c>
     </row>
@@ -5575,7 +5571,7 @@
         <v>240</v>
       </c>
       <c r="U14" s="11" t="str">
-        <f>DEC2BIN(T14,8)</f>
+        <f t="shared" si="1"/>
         <v>11110000</v>
       </c>
     </row>
@@ -5641,7 +5637,7 @@
         <v>224</v>
       </c>
       <c r="U15" s="11" t="str">
-        <f>DEC2BIN(T15,8)</f>
+        <f t="shared" si="1"/>
         <v>11100000</v>
       </c>
     </row>
@@ -5707,7 +5703,7 @@
         <v>192</v>
       </c>
       <c r="U16" s="11" t="str">
-        <f>DEC2BIN(T16,8)</f>
+        <f t="shared" si="1"/>
         <v>11000000</v>
       </c>
     </row>
@@ -5773,7 +5769,7 @@
         <v>128</v>
       </c>
       <c r="U17" s="11" t="str">
-        <f>DEC2BIN(T17,8)</f>
+        <f t="shared" si="1"/>
         <v>10000000</v>
       </c>
     </row>
@@ -5782,7 +5778,7 @@
         <v>0</v>
       </c>
       <c r="U18" s="11" t="str">
-        <f>DEC2BIN(T18,8)</f>
+        <f t="shared" si="1"/>
         <v>00000000</v>
       </c>
     </row>
@@ -5837,28 +5833,28 @@
         <v>39</v>
       </c>
       <c r="K21" s="46" t="str">
-        <f t="shared" ref="K21:K30" si="1">DEC2BIN(B21,8)</f>
+        <f t="shared" ref="K21:K30" si="2">DEC2BIN(B21,8)</f>
         <v>11000000</v>
       </c>
       <c r="L21" s="46" t="s">
         <v>57</v>
       </c>
       <c r="M21" s="46" t="str">
-        <f t="shared" ref="M21:M30" si="2">DEC2BIN(D21,8)</f>
+        <f t="shared" ref="M21:M30" si="3">DEC2BIN(D21,8)</f>
         <v>10101000</v>
       </c>
       <c r="N21" s="46" t="s">
         <v>57</v>
       </c>
       <c r="O21" s="46" t="str">
-        <f t="shared" ref="O21:O30" si="3">DEC2BIN(F21,8)</f>
+        <f t="shared" ref="O21:O30" si="4">DEC2BIN(F21,8)</f>
         <v>00000110</v>
       </c>
       <c r="P21" s="46" t="s">
         <v>57</v>
       </c>
       <c r="Q21" s="46" t="str">
-        <f t="shared" ref="Q21:Q30" si="4">DEC2BIN(H21,8)</f>
+        <f t="shared" ref="Q21:Q30" si="5">DEC2BIN(H21,8)</f>
         <v>00001101</v>
       </c>
     </row>
@@ -5892,28 +5888,28 @@
         <v>0</v>
       </c>
       <c r="K22" s="43" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>11000000</v>
       </c>
       <c r="L22" s="43" t="s">
         <v>57</v>
       </c>
       <c r="M22" s="43" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>10101000</v>
       </c>
       <c r="N22" s="43" t="s">
         <v>57</v>
       </c>
       <c r="O22" s="43" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>00000110</v>
       </c>
       <c r="P22" s="43" t="s">
         <v>57</v>
       </c>
       <c r="Q22" s="43" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>00000000</v>
       </c>
     </row>
@@ -5947,28 +5943,28 @@
         <v>39</v>
       </c>
       <c r="K23" s="46" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>11000000</v>
       </c>
       <c r="L23" s="46" t="s">
         <v>57</v>
       </c>
       <c r="M23" s="46" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>10101000</v>
       </c>
       <c r="N23" s="46" t="s">
         <v>57</v>
       </c>
       <c r="O23" s="46" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>00000111</v>
       </c>
       <c r="P23" s="46" t="s">
         <v>57</v>
       </c>
       <c r="Q23" s="46" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>00101001</v>
       </c>
     </row>
@@ -6004,28 +6000,28 @@
       <c r="I24"/>
       <c r="J24"/>
       <c r="K24" s="43" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>11000000</v>
       </c>
       <c r="L24" s="43" t="s">
         <v>57</v>
       </c>
       <c r="M24" s="43" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>10101000</v>
       </c>
       <c r="N24" s="43" t="s">
         <v>57</v>
       </c>
       <c r="O24" s="43" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>00000110</v>
       </c>
       <c r="P24" s="43" t="s">
         <v>57</v>
       </c>
       <c r="Q24" s="43" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>00000000</v>
       </c>
     </row>
@@ -6171,28 +6167,28 @@
         <v>39</v>
       </c>
       <c r="K27" s="45" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>00001010</v>
       </c>
       <c r="L27" s="45" t="s">
         <v>57</v>
       </c>
       <c r="M27" s="45" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>10101000</v>
       </c>
       <c r="N27" s="45" t="s">
         <v>57</v>
       </c>
       <c r="O27" s="45" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>00000001</v>
       </c>
       <c r="P27" s="45" t="s">
         <v>57</v>
       </c>
       <c r="Q27" s="45" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>00110011</v>
       </c>
     </row>
@@ -6228,28 +6224,28 @@
       <c r="I28" s="11"/>
       <c r="J28" s="11"/>
       <c r="K28" s="11" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>00001010</v>
       </c>
       <c r="L28" s="11" t="s">
         <v>57</v>
       </c>
       <c r="M28" s="11" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>10101000</v>
       </c>
       <c r="N28" s="11" t="s">
         <v>57</v>
       </c>
       <c r="O28" s="11" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>00000000</v>
       </c>
       <c r="P28" s="11" t="s">
         <v>57</v>
       </c>
       <c r="Q28" s="11" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>00000000</v>
       </c>
       <c r="V28" s="11"/>
@@ -6285,28 +6281,28 @@
         <v>39</v>
       </c>
       <c r="K29" s="45" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>11000000</v>
       </c>
       <c r="L29" s="45" t="s">
         <v>57</v>
       </c>
       <c r="M29" s="45" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>10101000</v>
       </c>
       <c r="N29" s="45" t="s">
         <v>57</v>
       </c>
       <c r="O29" s="45" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>00110010</v>
       </c>
       <c r="P29" s="45" t="s">
         <v>57</v>
       </c>
       <c r="Q29" s="45" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>00010111</v>
       </c>
     </row>
@@ -6342,28 +6338,28 @@
       <c r="I30"/>
       <c r="J30"/>
       <c r="K30" s="43" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>11000000</v>
       </c>
       <c r="L30" s="43" t="s">
         <v>57</v>
       </c>
       <c r="M30" s="43" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>10101000</v>
       </c>
       <c r="N30" s="43" t="s">
         <v>57</v>
       </c>
       <c r="O30" s="43" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>00110010</v>
       </c>
       <c r="P30" s="43" t="s">
         <v>57</v>
       </c>
       <c r="Q30" s="43" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>00000000</v>
       </c>
       <c r="S30"/>
@@ -6805,19 +6801,19 @@
         <v>0</v>
       </c>
       <c r="W18" s="58">
-        <f>IF(R8=R18,1,0)</f>
+        <f t="shared" ref="W18:Z19" si="1">IF(R8=R18,1,0)</f>
         <v>1</v>
       </c>
       <c r="X18" s="58">
-        <f>IF(S8=S18,1,0)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="Y18" s="58">
-        <f>IF(T8=T18,1,0)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="Z18" s="58">
-        <f>IF(U8=U18,1,0)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="AA18" s="58">
@@ -6877,19 +6873,19 @@
         <v>0</v>
       </c>
       <c r="W19" s="59">
-        <f>IF(R9=R19,1,0)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="X19" s="59">
-        <f>IF(S9=S19,1,0)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Y19" s="59">
-        <f>IF(T9=T19,1,0)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="Z19" s="59">
-        <f>IF(U9=U19,1,0)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="AA19" s="59">

</xml_diff>